<commit_message>
ver 0.4.1.3 minor correction
</commit_message>
<xml_diff>
--- a/data/datasetsinR.xlsx
+++ b/data/datasetsinR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kyowapharma-my.sharepoint.com/personal/araya-t_kyowayakuhin_co_jp/Documents/R_scripts/R入門/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R入門\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:40009_{7B23FD73-BEA6-497A-A12D-D53602F1DDCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E80609DA-691F-41A2-B855-71EE7DAEBEF9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89684EAD-02BC-4DB3-8659-9F1524185ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AirPassengers                  " sheetId="1" r:id="rId1"/>
@@ -1853,25 +1853,6 @@
     <phoneticPr fontId="18"/>
   </si>
   <si>
-    <t>睡眠薬2種を接種した学生の睡眠量のデータ</t>
-    <rPh sb="0" eb="3">
-      <t>スイミンヤク</t>
-    </rPh>
-    <rPh sb="4" eb="5">
-      <t>シュ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>セッシュ</t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t>ガクセイ</t>
-    </rPh>
-    <rPh sb="13" eb="16">
-      <t>スイミンリョウ</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
     <t>アンモニアをニトリル酸に酸化する工場のデータ</t>
     <rPh sb="10" eb="11">
       <t>サン</t>
@@ -2470,6 +2451,25 @@
     </rPh>
     <rPh sb="13" eb="15">
       <t>ヒョウコウ</t>
+    </rPh>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>睡眠薬2種を摂取した学生の睡眠量のデータ</t>
+    <rPh sb="0" eb="3">
+      <t>スイミンヤク</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>シュ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>セッシュ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ガクセイ</t>
+    </rPh>
+    <rPh sb="13" eb="16">
+      <t>スイミンリョウ</t>
     </rPh>
     <phoneticPr fontId="18"/>
   </si>
@@ -3186,9 +3186,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 テーマ">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3226,7 +3226,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3332,7 +3332,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3474,7 +3474,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3483,16 +3483,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E105"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="25.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="61.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="61.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>212</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3523,10 +3523,10 @@
         <v>166</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>167</v>
       </c>
@@ -3540,12 +3540,12 @@
         <v>166</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
@@ -3557,10 +3557,10 @@
         <v>166</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -3574,10 +3574,10 @@
         <v>169</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -3591,10 +3591,10 @@
         <v>169</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -3608,10 +3608,10 @@
         <v>169</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -3625,10 +3625,10 @@
         <v>169</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -3642,10 +3642,10 @@
         <v>166</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -3659,10 +3659,10 @@
         <v>169</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>177</v>
       </c>
@@ -3676,10 +3676,10 @@
         <v>179</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
@@ -3693,10 +3693,10 @@
         <v>181</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>182</v>
       </c>
@@ -3710,10 +3710,10 @@
         <v>181</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>18</v>
       </c>
@@ -3727,10 +3727,10 @@
         <v>169</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -3744,10 +3744,10 @@
         <v>169</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -3761,10 +3761,10 @@
         <v>166</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -3778,10 +3778,10 @@
         <v>166</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -3795,10 +3795,10 @@
         <v>169</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
@@ -3812,10 +3812,10 @@
         <v>169</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
@@ -3829,10 +3829,10 @@
         <v>166</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>32</v>
       </c>
@@ -3846,10 +3846,10 @@
         <v>169</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>34</v>
       </c>
@@ -3863,10 +3863,10 @@
         <v>169</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
@@ -3880,10 +3880,10 @@
         <v>169</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
@@ -3897,10 +3897,10 @@
         <v>169</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -3914,10 +3914,10 @@
         <v>166</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>42</v>
       </c>
@@ -3931,10 +3931,10 @@
         <v>169</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>44</v>
       </c>
@@ -3948,10 +3948,10 @@
         <v>199</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>46</v>
       </c>
@@ -3965,10 +3965,10 @@
         <v>169</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>48</v>
       </c>
@@ -3982,10 +3982,10 @@
         <v>179</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>50</v>
       </c>
@@ -3999,10 +3999,10 @@
         <v>166</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>51</v>
       </c>
@@ -4016,10 +4016,10 @@
         <v>166</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>53</v>
       </c>
@@ -4033,10 +4033,10 @@
         <v>166</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>55</v>
       </c>
@@ -4050,10 +4050,10 @@
         <v>169</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>57</v>
       </c>
@@ -4067,10 +4067,10 @@
         <v>169</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>59</v>
       </c>
@@ -4084,10 +4084,10 @@
         <v>218</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>61</v>
       </c>
@@ -4101,10 +4101,10 @@
         <v>209</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>219</v>
       </c>
@@ -4118,10 +4118,10 @@
         <v>218</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>64</v>
       </c>
@@ -4135,10 +4135,10 @@
         <v>166</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>66</v>
       </c>
@@ -4152,10 +4152,10 @@
         <v>218</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>68</v>
       </c>
@@ -4169,10 +4169,10 @@
         <v>181</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>70</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>72</v>
       </c>
@@ -4203,10 +4203,10 @@
         <v>169</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
         <v>74</v>
       </c>
@@ -4220,10 +4220,10 @@
         <v>169</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
         <v>76</v>
       </c>
@@ -4237,10 +4237,10 @@
         <v>169</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
         <v>78</v>
       </c>
@@ -4254,10 +4254,10 @@
         <v>169</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
         <v>80</v>
       </c>
@@ -4271,12 +4271,12 @@
         <v>166</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>82</v>
@@ -4288,12 +4288,12 @@
         <v>169</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A48" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>82</v>
@@ -4305,10 +4305,10 @@
         <v>169</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>83</v>
       </c>
@@ -4322,10 +4322,10 @@
         <v>169</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A50" s="1" t="s">
         <v>85</v>
       </c>
@@ -4339,10 +4339,10 @@
         <v>169</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A51" s="1" t="s">
         <v>87</v>
       </c>
@@ -4356,10 +4356,10 @@
         <v>166</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A52" s="1" t="s">
         <v>89</v>
       </c>
@@ -4373,10 +4373,10 @@
         <v>218</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A53" s="1" t="s">
         <v>91</v>
       </c>
@@ -4390,10 +4390,10 @@
         <v>166</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A54" s="1" t="s">
         <v>93</v>
       </c>
@@ -4407,10 +4407,10 @@
         <v>169</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A55" s="1" t="s">
         <v>95</v>
       </c>
@@ -4427,9 +4427,9 @@
         <v>238</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A56" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>96</v>
@@ -4444,7 +4444,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
         <v>97</v>
       </c>
@@ -4458,10 +4458,10 @@
         <v>209</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A58" s="1" t="s">
         <v>98</v>
       </c>
@@ -4475,10 +4475,10 @@
         <v>169</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>101</v>
       </c>
@@ -4492,12 +4492,12 @@
         <v>169</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A60" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>102</v>
@@ -4509,12 +4509,12 @@
         <v>218</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>102</v>
@@ -4526,10 +4526,10 @@
         <v>166</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A62" s="1" t="s">
         <v>103</v>
       </c>
@@ -4543,10 +4543,10 @@
         <v>169</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A63" s="1" t="s">
         <v>105</v>
       </c>
@@ -4560,10 +4560,10 @@
         <v>169</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
         <v>107</v>
       </c>
@@ -4577,10 +4577,10 @@
         <v>179</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A65" s="1" t="s">
         <v>108</v>
       </c>
@@ -4594,12 +4594,12 @@
         <v>237</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A66" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>100</v>
@@ -4611,12 +4611,12 @@
         <v>166</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A67" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>100</v>
@@ -4628,12 +4628,12 @@
         <v>166</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>100</v>
@@ -4645,10 +4645,10 @@
         <v>166</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A69" s="1" t="s">
         <v>110</v>
       </c>
@@ -4662,10 +4662,10 @@
         <v>166</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A70" s="1" t="s">
         <v>112</v>
       </c>
@@ -4679,10 +4679,10 @@
         <v>169</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>114</v>
       </c>
@@ -4696,10 +4696,10 @@
         <v>166</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A72" s="1" t="s">
         <v>116</v>
       </c>
@@ -4713,10 +4713,10 @@
         <v>169</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A73" s="1" t="s">
         <v>118</v>
       </c>
@@ -4730,10 +4730,10 @@
         <v>169</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A74" s="1" t="s">
         <v>120</v>
       </c>
@@ -4747,10 +4747,10 @@
         <v>166</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A75" s="1" t="s">
         <v>122</v>
       </c>
@@ -4764,10 +4764,10 @@
         <v>166</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A76" s="1" t="s">
         <v>124</v>
       </c>
@@ -4781,10 +4781,10 @@
         <v>169</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A77" s="1" t="s">
         <v>126</v>
       </c>
@@ -4798,10 +4798,10 @@
         <v>218</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>128</v>
       </c>
@@ -4815,10 +4815,10 @@
         <v>237</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A79" s="1" t="s">
         <v>130</v>
       </c>
@@ -4832,10 +4832,10 @@
         <v>166</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A80" s="1" t="s">
         <v>132</v>
       </c>
@@ -4849,10 +4849,10 @@
         <v>169</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A81" s="1" t="s">
         <v>134</v>
       </c>
@@ -4869,7 +4869,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A82" s="1" t="s">
         <v>136</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A83" s="1" t="s">
         <v>138</v>
       </c>
@@ -4900,10 +4900,10 @@
         <v>237</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A84" s="1" t="s">
         <v>140</v>
       </c>
@@ -4917,10 +4917,10 @@
         <v>169</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A85" s="1" t="s">
         <v>142</v>
       </c>
@@ -4928,16 +4928,16 @@
         <v>143</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>265</v>
+        <v>366</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A86" s="1" t="s">
         <v>145</v>
       </c>
@@ -4945,186 +4945,186 @@
         <v>144</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A87" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>144</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>144</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>218</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A89" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A90" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A91" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>181</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A93" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A94" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A95" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A96" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>147</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>166</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A97" s="1" t="s">
         <v>148</v>
       </c>
@@ -5132,33 +5132,33 @@
         <v>149</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>166</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A98" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>150</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>166</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A99" s="1" t="s">
         <v>151</v>
       </c>
@@ -5166,16 +5166,16 @@
         <v>152</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A100" s="1" t="s">
         <v>153</v>
       </c>
@@ -5183,16 +5183,16 @@
         <v>154</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>166</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A101" s="1" t="s">
         <v>155</v>
       </c>
@@ -5200,16 +5200,16 @@
         <v>156</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A102" s="1" t="s">
         <v>157</v>
       </c>
@@ -5217,16 +5217,16 @@
         <v>158</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D102" s="1" t="s">
         <v>166</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A103" s="1" t="s">
         <v>159</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>160</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>218</v>
@@ -5243,7 +5243,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A104" s="1" t="s">
         <v>161</v>
       </c>
@@ -5251,16 +5251,16 @@
         <v>162</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D104" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A105" s="1" t="s">
         <v>163</v>
       </c>
@@ -5268,13 +5268,13 @@
         <v>164</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>169</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>